<commit_message>
publish: sync from 正本 2026-09-25T12:41:45Z
</commit_message>
<xml_diff>
--- a/plugins/osi-finance/assets/templates/支払管理台帳_テンプレート.xlsx
+++ b/plugins/osi-finance/assets/templates/支払管理台帳_テンプレート.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -510,31 +510,38 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>・月次支払管理＝支払の実績。月次支払スケジュール＝契約から展開した支払の予定。経費一覧＝明細の蓄積（ここから仕訳を起こさない）。</t>
+          <t>・受領請求書を月次支払管理に起票するときは 受領請求書ファイル（01.受領請求書/YYYY-MM/…pdf）を必ず書きます。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>・月次支払管理＝支払の実績。月次支払スケジュール＝契約から展開した支払の予定。経費一覧＝明細の蓄積（ここから仕訳を起こさない）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>・源泉徴収管理：源泉対象の支払の税額と納付状況。</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>記入例（参考。台帳には書かない）</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  支払先マスタ：支払先ID=V-001 / 支払先名=サンプル株式会社 / 支払先区分=法人 / 支払カテゴリ=外注費 / 取引先ID=P-001 / 既定の支払方法=振込 / 源泉徴収対象=なし / ステータス=支払対象</t>
+          <t>記入例（参考。台帳には書かない）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  支払先マスタ：支払先ID=V-001 / 支払カテゴリ=外注費 / 取引先ID=P-001 / 既定の支払方法=振込 / 源泉徴収対象=なし / ステータス=支払対象</t>
         </is>
       </c>
     </row>
@@ -549,36 +556,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AA3"/>
+  <dimension ref="A2:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="3" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="3" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" style="3" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" style="3" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" style="3" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="10" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -596,130 +601,120 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>支払先名</t>
+          <t>支払先区分</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>支払先区分</t>
+          <t>支払カテゴリ</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>支払カテゴリ</t>
+          <t>メールアドレス</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>主担当者名</t>
+          <t>振込先銀行</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>メールアドレス</t>
+          <t>振込先支店</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>振込先銀行</t>
+          <t>口座種別</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>振込先支店</t>
+          <t>口座番号</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>口座種別</t>
+          <t>口座名義</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>口座番号</t>
+          <t>契約開始日</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>口座名義</t>
+          <t>契約終了日</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>契約開始日</t>
+          <t>契約タイプ</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>契約終了日</t>
+          <t>月額固定（税抜）</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>契約タイプ</t>
+          <t>時間単価（税抜）</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>月額固定（税抜）</t>
+          <t>消費税率</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>時間単価（税抜）</t>
+          <t>源泉徴収対象</t>
         </is>
       </c>
       <c r="Q3" s="4" t="inlineStr">
         <is>
-          <t>消費税率</t>
+          <t>源泉徴収税率</t>
         </is>
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>源泉徴収対象</t>
+          <t>支払サイクル</t>
         </is>
       </c>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>源泉徴収税率</t>
+          <t>取引先ID</t>
         </is>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>支払サイクル</t>
+          <t>ステータス</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>取引先ID</t>
+          <t>作成者</t>
         </is>
       </c>
       <c r="V3" s="4" t="inlineStr">
         <is>
-          <t>ステータス</t>
+          <t>作成日時</t>
         </is>
       </c>
       <c r="W3" s="4" t="inlineStr">
         <is>
-          <t>作成者</t>
+          <t>更新者</t>
         </is>
       </c>
       <c r="X3" s="4" t="inlineStr">
         <is>
-          <t>作成日時</t>
+          <t>更新日時</t>
         </is>
       </c>
       <c r="Y3" s="4" t="inlineStr">
-        <is>
-          <t>更新者</t>
-        </is>
-      </c>
-      <c r="Z3" s="4" t="inlineStr">
-        <is>
-          <t>更新日時</t>
-        </is>
-      </c>
-      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>既定の支払方法</t>
         </is>
@@ -727,19 +722,19 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="C4:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+    <dataValidation sqref="B4:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"法人,個人,個人事業主,要確認"</formula1>
     </dataValidation>
-    <dataValidation sqref="N4:N2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+    <dataValidation sqref="L4:L2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"月額固定,都度"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q4:Q2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+    <dataValidation sqref="O4:O2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"10.0%,0.0%,非課税,対象外（不課税）"</formula1>
     </dataValidation>
-    <dataValidation sqref="V4:V2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+    <dataValidation sqref="T4:T2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"支払対象,要確認"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA4:AA2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+    <dataValidation sqref="Y4:Y2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"振込,カード,口座振替,現金,カード発行会社"</formula1>
     </dataValidation>
   </dataValidations>
@@ -753,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:AB4"/>
+  <dimension ref="A4:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="3" min="1" max="1"/>
@@ -784,6 +779,9 @@
     <col width="10" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="4">
@@ -927,9 +925,24 @@
           <t>支払方法</t>
         </is>
       </c>
+      <c r="AC4" s="4" t="inlineStr">
+        <is>
+          <t>突合結果</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>突合日時</t>
+        </is>
+      </c>
+      <c r="AE4" s="4" t="inlineStr">
+        <is>
+          <t>受領請求書ファイル</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="C5:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"外注費,経費,その他"</formula1>
     </dataValidation>
@@ -938,6 +951,9 @@
     </dataValidation>
     <dataValidation sqref="AB5:AB2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
       <formula1>"振込,カード,口座振替,現金"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC5:AC2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"一致,未計上"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>